<commit_message>
Update wedding website schedule and typography styles
</commit_message>
<xml_diff>
--- a/data/rsvps.xlsx
+++ b/data/rsvps.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="40350" yWindow="1635" windowWidth="22710" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVPs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -50,7 +49,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -461,7 +460,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-01 22:49:00</t>
+          <t>2026-07-04 15:13:55</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,17 +490,12 @@
       </c>
       <c r="G2" t="n">
         <v>2</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-01 19:29:18</t>
+          <t>2026-07-04 18:07:25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -521,12 +515,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Hindu Wedding Ceremony</t>
+          <t>Traditional Telugu Wedding</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -541,7 +535,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-01 19:02:31</t>
+          <t>2026-07-04 17:31:40</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -561,7 +555,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Christian Wedding &amp; Reception</t>
+          <t>Church Wedding and Reception</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">

</xml_diff>

<commit_message>
updates the schedule tab
</commit_message>
<xml_diff>
--- a/data/rsvps.xlsx
+++ b/data/rsvps.xlsx
@@ -460,7 +460,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:13:55</t>
+          <t>2026-07-06 21:24:04</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -490,6 +490,11 @@
       </c>
       <c r="G2" t="n">
         <v>2</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -535,7 +540,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-04 17:31:40</t>
+          <t>2026-07-06 21:09:59</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -565,6 +570,11 @@
       </c>
       <c r="G4" t="n">
         <v>2</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>